<commit_message>
add cucumber feature files
</commit_message>
<xml_diff>
--- a/MyntraDemo/src/test/resources/testdata (1).xlsx
+++ b/MyntraDemo/src/test/resources/testdata (1).xlsx
@@ -1,21 +1,18 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29822"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
-  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
-    <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\HP\Documents\"/>
-    </mc:Choice>
-  </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC60CC38-4BCF-404F-AEF3-D6234388E565}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:801_{A21B5AF5-71DE-499F-B02B-54206F4FFB08}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="FilterData" sheetId="1" r:id="rId1"/>
+    <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="0"/>
+  <oleSize ref="A1:O10"/>
 </workbook>
 </file>
 
@@ -416,4 +413,13 @@
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BEC866DC-F2F0-4AFF-AD5F-B4DF49844840}">
+  <dimension ref="A1"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>